<commit_message>
fix(pizza-shop-checklists-en): ronda 1 de la revisión adversarial — 2 MAYOR + 21 menor aplicados
National Pizza Day, Pi Day y National Pizza Month en el calendario; objetivo de horno según el tipo (deck/conveyor
vs napolitano) y harina high-gluten; ceniza al día siguiente a 3 ft; orden campana-horno; porciones con
procedimiento 3-501.19; no servir a visiblemente ebrios; kilometraje del repartidor (29 CFR 531.35); mínimos
de inventario en formatos de compra US. Landing alineada. 4 hermanos idénticos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/pizza-shop-checklist-templates/01-pizza-shop-opening-closing-checklists.xlsx
+++ b/astro-site/public/dl/pizza-shop-checklist-templates/01-pizza-shop-opening-closing-checklists.xlsx
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>Pizza maker</t>
+          <t>Shift manager</t>
         </is>
       </c>
       <c r="E10" s="27" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B16" s="34" t="inlineStr">
         <is>
-          <t>Check oven temp: 750–840 °F (Neapolitan) — log reading: ____ °F</t>
+          <t>Check oven temp against your oven's target (wood-fired Neapolitan 750–840 °F; gas deck, conveyor or electric: per your recipe and manufacturer) — target: ____ °F · reading: ____ °F</t>
         </is>
       </c>
       <c r="C16" s="27" t="inlineStr">
@@ -1526,9 +1526,9 @@
       <c r="A31" s="29" t="n">
         <v>23</v>
       </c>
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t>Check flour stock (00, whole wheat)</t>
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>Check flour stock (00, high-gluten or bread flour, whole wheat)</t>
         </is>
       </c>
       <c r="C31" s="27" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="B10" s="33" t="inlineStr">
         <is>
-          <t>Date-mark everything: ready-to-eat food keeps 7 days at 41 °F, prep day = day 1 (FDA 3-501.17)</t>
+          <t>Date-mark ready-to-eat TCS food kept over 24 h: 7 days max at 41 °F or below, prep day = day 1 (FDA 3-501.17)</t>
         </is>
       </c>
       <c r="C10" s="27" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>Remove ash only when cold (at close, or first thing next morning) into a lidded METAL container, never trash or plastic (NFPA 96)</t>
+          <t>Ash: never take it out hot at close; remove it cold, usually first thing next morning before lighting, into a closed METAL container kept at least 3 ft from the oven, never trash or plastic (NFPA 96)</t>
         </is>
       </c>
       <c r="C13" s="27" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="E13" s="27" t="inlineStr">
         <is>
-          <t>11:00 PM</t>
+          <t>Next AM</t>
         </is>
       </c>
       <c r="F13" s="28" t="n"/>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="B15" s="34" t="inlineStr">
         <is>
-          <t>Turn off the exhaust hood (wood-fired oven: not while fire or embers remain; follow the manufacturers)</t>
+          <t>Turn off the exhaust hood (wood-fired oven: not while fire or embers remain; follow the oven and hood manufacturers' instructions)</t>
         </is>
       </c>
       <c r="C15" s="27" t="inlineStr">

</xml_diff>